<commit_message>
updated Sankey diagram with new SES AS.
</commit_message>
<xml_diff>
--- a/Data/Table_Discussion.xlsx
+++ b/Data/Table_Discussion.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexandrabl/Desktop/MarEEchange/1_Paper_publi/1_SES/R/prOACT_pathways/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8851BA8C-810B-CB40-86BD-F80EC4723A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E877724B-F5DB-994E-B61C-421E52FCA6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="23500" xr2:uid="{714A1C6C-974B-1E4A-9034-5DDE98B770F7}"/>
+    <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{714A1C6C-974B-1E4A-9034-5DDE98B770F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$1</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="37">
   <si>
     <t>Alternatives</t>
   </si>
@@ -134,32 +137,36 @@
     <t>s_f_environmentally_friendly</t>
   </si>
   <si>
-    <t>S_AS_rule_making</t>
-  </si>
-  <si>
     <t>S_AS_scientific_advice</t>
   </si>
   <si>
     <t>SE_AS_harvesting</t>
   </si>
   <si>
-    <t>S_AS_socio_economic</t>
-  </si>
-  <si>
     <t>E_AS_predation</t>
   </si>
   <si>
     <t>PE_AS_abiotic</t>
+  </si>
+  <si>
+    <t>S_AS_mismanagement</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -185,8 +192,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -549,7 +557,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -560,7 +568,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -571,7 +579,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -582,7 +590,7 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -593,7 +601,7 @@
         <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -604,7 +612,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -615,7 +623,7 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -626,7 +634,7 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -637,7 +645,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -648,7 +656,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -659,7 +667,7 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -670,7 +678,7 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -681,7 +689,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -692,7 +700,7 @@
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -703,7 +711,7 @@
         <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -714,7 +722,7 @@
         <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -725,7 +733,7 @@
         <v>19</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -736,7 +744,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -747,7 +755,7 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -758,7 +766,7 @@
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -769,7 +777,7 @@
         <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -780,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -791,7 +799,7 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -802,7 +810,7 @@
         <v>20</v>
       </c>
       <c r="C25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -813,7 +821,7 @@
         <v>6</v>
       </c>
       <c r="C26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -824,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -834,8 +842,8 @@
       <c r="B28" t="s">
         <v>14</v>
       </c>
-      <c r="C28" t="s">
-        <v>35</v>
+      <c r="C28" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -846,7 +854,7 @@
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -856,8 +864,8 @@
       <c r="B30" t="s">
         <v>23</v>
       </c>
-      <c r="C30" t="s">
-        <v>35</v>
+      <c r="C30" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -867,8 +875,8 @@
       <c r="B31" t="s">
         <v>16</v>
       </c>
-      <c r="C31" t="s">
-        <v>35</v>
+      <c r="C31" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -878,8 +886,8 @@
       <c r="B32" t="s">
         <v>12</v>
       </c>
-      <c r="C32" t="s">
-        <v>35</v>
+      <c r="C32" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -890,7 +898,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -901,7 +909,7 @@
         <v>15</v>
       </c>
       <c r="C34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -912,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -922,8 +930,8 @@
       <c r="B36" t="s">
         <v>21</v>
       </c>
-      <c r="C36" t="s">
-        <v>35</v>
+      <c r="C36" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -934,7 +942,7 @@
         <v>9</v>
       </c>
       <c r="C37" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -944,8 +952,8 @@
       <c r="B38" t="s">
         <v>23</v>
       </c>
-      <c r="C38" t="s">
-        <v>35</v>
+      <c r="C38" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -956,7 +964,7 @@
         <v>6</v>
       </c>
       <c r="C39" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -967,7 +975,7 @@
         <v>22</v>
       </c>
       <c r="C40" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -978,7 +986,7 @@
         <v>15</v>
       </c>
       <c r="C41" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -989,7 +997,7 @@
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1000,7 +1008,7 @@
         <v>13</v>
       </c>
       <c r="C43" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -1011,7 +1019,7 @@
         <v>11</v>
       </c>
       <c r="C44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -1022,10 +1030,11 @@
         <v>6</v>
       </c>
       <c r="C45" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{74B3850C-E65A-1944-A60F-6755105C59A4}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>